<commit_message>
NPB自動更新(1軍): 2026-09-14 (steps: all)
</commit_message>
<xml_diff>
--- a/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-14.xlsx
+++ b/data/プロ野球/2026年/1軍/レギュラーシーズン/games/datamart/2026-09-14.xlsx
@@ -84121,7 +84121,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>9回106球4安打7奪三振無失点の完封勝利。圧倒的な投球でチームを勝利に導いた。</t>
+          <t>9回を投げ被安打4、7奪三振の完封勝利。相手打線を完璧に封じ込めた。</t>
         </is>
       </c>
     </row>
@@ -84136,17 +84136,17 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>古市 尊</t>
+          <t>細川 成也</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>DeNA</t>
+          <t>中日</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>12回裏、犠打失策でサヨナラ勝ちを呼び込んだ。延長戦の激闘に終止符を打った。</t>
+          <t>1回表にレフトスタンドへ先制2ランを放ち、チームの勝利に貢献した。</t>
         </is>
       </c>
     </row>
@@ -84161,17 +84161,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>大城 卓三</t>
+          <t>牧 秀悟</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>巨人</t>
+          <t>DeNA</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5回表、ランナー三塁からライトスタンドへの2ランで試合を同点に戻した。</t>
+          <t>1回裏にレフトスタンドへ先制ソロホームランを放ち、チームに勢いをつけた。</t>
         </is>
       </c>
     </row>
@@ -84186,17 +84186,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>細川 成也</t>
+          <t>大城 卓三</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>中日</t>
+          <t>巨人</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1回表、フルカウントからレフトスタンドへ先制2ランを放ち、試合の主導権を握った。</t>
+          <t>5回表に同点2ランホームランを放ち、試合の流れを大きく引き寄せた。</t>
         </is>
       </c>
     </row>
@@ -84211,17 +84211,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>牧 秀悟</t>
+          <t>増田 陸</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>DeNA</t>
+          <t>巨人</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1回裏、カウント2-0からレフトスタンドへ先制ホームランを放ち、チームに勢いを与えた。</t>
+          <t>6回表に勝ち越しホームランを放ち、チームにリードをもたらす一打となった。</t>
         </is>
       </c>
     </row>
@@ -84236,17 +84236,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>泉口 友汰</t>
+          <t>モンテロ</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>巨人</t>
+          <t>広島</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>5打数4安打の猛打賞を記録し、打線の中核として攻撃を牽引した。</t>
+          <t>7回表にバックスクリーンへダメ押しソロを放ち、リードを広げ勝利を決定づけた。</t>
         </is>
       </c>
     </row>

</xml_diff>